<commit_message>
chore: Update DATA SIJAKA.xlsx.
</commit_message>
<xml_diff>
--- a/DATA SIJAKA.xlsx
+++ b/DATA SIJAKA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abichoy/Documents/sijakadev2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1404328-CE36-ED47-9CA3-ECAD135D287E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00D9814-D369-FE47-86E0-F530A505C7D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3980" yWindow="2780" windowWidth="28040" windowHeight="17180" activeTab="1" xr2:uid="{735AD8D3-2DA3-3647-978F-3D3AB67DDBE0}"/>
+    <workbookView xWindow="-360" yWindow="4320" windowWidth="28040" windowHeight="17180" xr2:uid="{735AD8D3-2DA3-3647-978F-3D3AB67DDBE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Kapal" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="164">
   <si>
     <t>Kode Jaket</t>
   </si>
@@ -494,6 +494,42 @@
   </si>
   <si>
     <t>Kontak</t>
+  </si>
+  <si>
+    <t>0882019047357</t>
+  </si>
+  <si>
+    <t>085342082925</t>
+  </si>
+  <si>
+    <t>0'85240455235</t>
+  </si>
+  <si>
+    <t>085143605857</t>
+  </si>
+  <si>
+    <t>087778325691</t>
+  </si>
+  <si>
+    <t>082188515446</t>
+  </si>
+  <si>
+    <t>08114409743</t>
+  </si>
+  <si>
+    <t>085230812696</t>
+  </si>
+  <si>
+    <t>085342574099</t>
+  </si>
+  <si>
+    <t>085340697154</t>
+  </si>
+  <si>
+    <t>085298470644</t>
+  </si>
+  <si>
+    <t>085255822441</t>
   </si>
 </sst>
 </file>
@@ -509,13 +545,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
@@ -524,6 +553,12 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -570,7 +605,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -579,16 +614,17 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1273,8 +1309,8 @@
       <c r="D3" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="E3" s="3">
-        <v>85342082925</v>
+      <c r="E3" s="7" t="s">
+        <v>153</v>
       </c>
       <c r="F3" s="3"/>
     </row>
@@ -1288,8 +1324,8 @@
       <c r="D4" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="3">
-        <v>882019047357</v>
+      <c r="E4" s="7" t="s">
+        <v>152</v>
       </c>
       <c r="F4" s="3"/>
     </row>
@@ -1300,7 +1336,7 @@
       <c r="C5" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="8" t="s">
         <v>147</v>
       </c>
       <c r="E5" s="3" t="s">
@@ -1333,8 +1369,8 @@
       <c r="D7" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="E7" s="3">
-        <v>85240455235</v>
+      <c r="E7" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="F7" s="3"/>
     </row>
@@ -1348,8 +1384,8 @@
       <c r="D8" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E8" s="3">
-        <v>85143605857</v>
+      <c r="E8" s="7" t="s">
+        <v>155</v>
       </c>
       <c r="F8" s="3"/>
     </row>
@@ -1363,8 +1399,8 @@
       <c r="D9" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E9" s="3">
-        <v>82188515446</v>
+      <c r="E9" s="7" t="s">
+        <v>157</v>
       </c>
       <c r="F9" s="3"/>
     </row>
@@ -1378,8 +1414,8 @@
       <c r="D10" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="E10" s="3">
-        <v>87778325691</v>
+      <c r="E10" s="7" t="s">
+        <v>156</v>
       </c>
       <c r="F10" s="3"/>
     </row>
@@ -1393,8 +1429,8 @@
       <c r="D11" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="E11" s="3">
-        <v>8114409743</v>
+      <c r="E11" s="7" t="s">
+        <v>158</v>
       </c>
       <c r="F11" s="3"/>
     </row>
@@ -1408,8 +1444,8 @@
       <c r="D12" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="E12" s="3">
-        <v>85230812696</v>
+      <c r="E12" s="7" t="s">
+        <v>159</v>
       </c>
       <c r="F12" s="3"/>
     </row>
@@ -1423,8 +1459,8 @@
       <c r="D13" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="E13" s="3">
-        <v>85342574099</v>
+      <c r="E13" s="7" t="s">
+        <v>160</v>
       </c>
       <c r="F13" s="3"/>
     </row>
@@ -1438,8 +1474,8 @@
       <c r="D14" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E14" s="3">
-        <v>85340697154</v>
+      <c r="E14" s="7" t="s">
+        <v>161</v>
       </c>
       <c r="F14" s="3"/>
     </row>
@@ -1450,11 +1486,11 @@
       <c r="C15" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="E15" s="3">
-        <v>85298470644</v>
+      <c r="E15" s="7" t="s">
+        <v>162</v>
       </c>
       <c r="F15" s="3"/>
     </row>
@@ -1468,8 +1504,8 @@
       <c r="D16" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="E16" s="3">
-        <v>85255822441</v>
+      <c r="E16" s="7" t="s">
+        <v>163</v>
       </c>
       <c r="F16" s="3"/>
     </row>
@@ -3621,7 +3657,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C5:H104">
     <sortCondition ref="C4:C104"/>
   </sortState>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>